<commit_message>
Expand Cameroon diagnostics and WBES analysis
Add Census and administrative robustness checks, BDF asset diagnostics, WBES exporter interactions, updated generated outputs and slides, B-READY mapping scaffolding, and cumulative project documentation.
</commit_message>
<xml_diff>
--- a/docs/reference/cmr_census_activity_nacam_crosswalk.xlsx
+++ b/docs/reference/cmr_census_activity_nacam_crosswalk.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3017" uniqueCount="987">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="995">
   <si>
     <t>citi_branch</t>
   </si>
@@ -2974,6 +2974,30 @@
   </si>
   <si>
     <t>Broadcast labels map to the current post/telecom branch.</t>
+  </si>
+  <si>
+    <t>Industrial/export agriculture</t>
+  </si>
+  <si>
+    <t>Services mainly to enterprises</t>
+  </si>
+  <si>
+    <t>Post/telecommunications</t>
+  </si>
+  <si>
+    <t>Accommodation/food services</t>
+  </si>
+  <si>
+    <t>Wholesale and retail trade</t>
+  </si>
+  <si>
+    <t>Wholesale/retail trade</t>
+  </si>
+  <si>
+    <t>Electricity/water supply</t>
+  </si>
+  <si>
+    <t>Wholesale/retail</t>
   </si>
 </sst>
 </file>
@@ -3018,7 +3042,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:N274"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -3098,7 +3122,7 @@
         <v>585</v>
       </c>
       <c r="K2" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="L2" s="1">
         <v>0</v>
@@ -3142,7 +3166,7 @@
         <v>585</v>
       </c>
       <c r="K3" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="L3" s="1">
         <v>0</v>
@@ -3186,7 +3210,7 @@
         <v>586</v>
       </c>
       <c r="K4" t="s">
-        <v>733</v>
+        <v>987</v>
       </c>
       <c r="L4" s="1">
         <v>0</v>
@@ -3230,7 +3254,7 @@
         <v>586</v>
       </c>
       <c r="K5" t="s">
-        <v>733</v>
+        <v>987</v>
       </c>
       <c r="L5" s="1">
         <v>0</v>
@@ -3274,7 +3298,7 @@
         <v>587</v>
       </c>
       <c r="K6" t="s">
-        <v>734</v>
+        <v>727</v>
       </c>
       <c r="L6" s="1">
         <v>0</v>
@@ -3318,7 +3342,7 @@
         <v>588</v>
       </c>
       <c r="K7" t="s">
-        <v>735</v>
+        <v>987</v>
       </c>
       <c r="L7" s="1">
         <v>0</v>
@@ -3362,7 +3386,7 @@
         <v>588</v>
       </c>
       <c r="K8" t="s">
-        <v>735</v>
+        <v>987</v>
       </c>
       <c r="L8" s="1">
         <v>0</v>
@@ -3406,7 +3430,7 @@
         <v>589</v>
       </c>
       <c r="K9" t="s">
-        <v>736</v>
+        <v>727</v>
       </c>
       <c r="L9" s="1">
         <v>0</v>
@@ -3450,7 +3474,7 @@
         <v>590</v>
       </c>
       <c r="K10" t="s">
-        <v>737</v>
+        <v>987</v>
       </c>
       <c r="L10" s="1">
         <v>0</v>
@@ -3494,7 +3518,7 @@
         <v>590</v>
       </c>
       <c r="K11" t="s">
-        <v>737</v>
+        <v>987</v>
       </c>
       <c r="L11" s="1">
         <v>0</v>
@@ -3538,7 +3562,7 @@
         <v>590</v>
       </c>
       <c r="K12" t="s">
-        <v>737</v>
+        <v>987</v>
       </c>
       <c r="L12" s="1">
         <v>0</v>
@@ -3582,7 +3606,7 @@
         <v>591</v>
       </c>
       <c r="K13" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="L13" s="1">
         <v>0</v>
@@ -3626,7 +3650,7 @@
         <v>591</v>
       </c>
       <c r="K14" t="s">
-        <v>738</v>
+        <v>727</v>
       </c>
       <c r="L14" s="1">
         <v>0</v>
@@ -3670,7 +3694,7 @@
         <v>592</v>
       </c>
       <c r="K15" t="s">
-        <v>739</v>
+        <v>987</v>
       </c>
       <c r="L15" s="1">
         <v>1</v>
@@ -3758,7 +3782,7 @@
         <v>594</v>
       </c>
       <c r="K17" t="s">
-        <v>741</v>
+        <v>988</v>
       </c>
       <c r="L17" s="1">
         <v>0</v>
@@ -3802,7 +3826,7 @@
         <v>594</v>
       </c>
       <c r="K18" t="s">
-        <v>741</v>
+        <v>988</v>
       </c>
       <c r="L18" s="1">
         <v>0</v>
@@ -3976,7 +4000,7 @@
         <v>598</v>
       </c>
       <c r="K22" t="s">
-        <v>745</v>
+        <v>988</v>
       </c>
       <c r="L22" s="1">
         <v>0</v>
@@ -4020,7 +4044,7 @@
         <v>598</v>
       </c>
       <c r="K23" t="s">
-        <v>745</v>
+        <v>988</v>
       </c>
       <c r="L23" s="1">
         <v>0</v>
@@ -4148,7 +4172,7 @@
         <v>601</v>
       </c>
       <c r="K26" t="s">
-        <v>748</v>
+        <v>988</v>
       </c>
       <c r="L26" s="1">
         <v>0</v>
@@ -4498,7 +4522,7 @@
         <v>606</v>
       </c>
       <c r="K34" t="s">
-        <v>753</v>
+        <v>988</v>
       </c>
       <c r="L34" s="1">
         <v>0</v>
@@ -4762,7 +4786,7 @@
         <v>610</v>
       </c>
       <c r="K40" t="s">
-        <v>757</v>
+        <v>988</v>
       </c>
       <c r="L40" s="1">
         <v>0</v>
@@ -4806,7 +4830,7 @@
         <v>610</v>
       </c>
       <c r="K41" t="s">
-        <v>757</v>
+        <v>988</v>
       </c>
       <c r="L41" s="1">
         <v>0</v>
@@ -4938,7 +4962,7 @@
         <v>612</v>
       </c>
       <c r="K44" t="s">
-        <v>759</v>
+        <v>988</v>
       </c>
       <c r="L44" s="1">
         <v>0</v>
@@ -5026,7 +5050,7 @@
         <v>614</v>
       </c>
       <c r="K46" t="s">
-        <v>761</v>
+        <v>988</v>
       </c>
       <c r="L46" s="1">
         <v>0</v>
@@ -5070,7 +5094,7 @@
         <v>614</v>
       </c>
       <c r="K47" t="s">
-        <v>761</v>
+        <v>988</v>
       </c>
       <c r="L47" s="1">
         <v>0</v>
@@ -5158,7 +5182,7 @@
         <v>616</v>
       </c>
       <c r="K49" t="s">
-        <v>763</v>
+        <v>988</v>
       </c>
       <c r="L49" s="1">
         <v>0</v>
@@ -5378,7 +5402,7 @@
         <v>619</v>
       </c>
       <c r="K54" t="s">
-        <v>766</v>
+        <v>988</v>
       </c>
       <c r="L54" s="1">
         <v>0</v>
@@ -5422,7 +5446,7 @@
         <v>619</v>
       </c>
       <c r="K55" t="s">
-        <v>766</v>
+        <v>988</v>
       </c>
       <c r="L55" s="1">
         <v>0</v>
@@ -5510,7 +5534,7 @@
         <v>621</v>
       </c>
       <c r="K57" t="s">
-        <v>768</v>
+        <v>988</v>
       </c>
       <c r="L57" s="1">
         <v>0</v>
@@ -5774,7 +5798,7 @@
         <v>624</v>
       </c>
       <c r="K63" t="s">
-        <v>771</v>
+        <v>988</v>
       </c>
       <c r="L63" s="1">
         <v>0</v>
@@ -5818,7 +5842,7 @@
         <v>624</v>
       </c>
       <c r="K64" t="s">
-        <v>771</v>
+        <v>988</v>
       </c>
       <c r="L64" s="1">
         <v>0</v>
@@ -5862,7 +5886,7 @@
         <v>624</v>
       </c>
       <c r="K65" t="s">
-        <v>771</v>
+        <v>988</v>
       </c>
       <c r="L65" s="1">
         <v>0</v>
@@ -5906,7 +5930,7 @@
         <v>624</v>
       </c>
       <c r="K66" t="s">
-        <v>771</v>
+        <v>988</v>
       </c>
       <c r="L66" s="1">
         <v>0</v>
@@ -6170,7 +6194,7 @@
         <v>629</v>
       </c>
       <c r="K72" t="s">
-        <v>776</v>
+        <v>988</v>
       </c>
       <c r="L72" s="1">
         <v>0</v>
@@ -6214,7 +6238,7 @@
         <v>630</v>
       </c>
       <c r="K73" t="s">
-        <v>777</v>
+        <v>989</v>
       </c>
       <c r="L73" s="1">
         <v>0</v>
@@ -6258,7 +6282,7 @@
         <v>631</v>
       </c>
       <c r="K74" t="s">
-        <v>778</v>
+        <v>988</v>
       </c>
       <c r="L74" s="1">
         <v>0</v>
@@ -6302,7 +6326,7 @@
         <v>631</v>
       </c>
       <c r="K75" t="s">
-        <v>778</v>
+        <v>988</v>
       </c>
       <c r="L75" s="1">
         <v>0</v>
@@ -6346,7 +6370,7 @@
         <v>631</v>
       </c>
       <c r="K76" t="s">
-        <v>778</v>
+        <v>988</v>
       </c>
       <c r="L76" s="1">
         <v>0</v>
@@ -6566,7 +6590,7 @@
         <v>635</v>
       </c>
       <c r="K81" t="s">
-        <v>782</v>
+        <v>988</v>
       </c>
       <c r="L81" s="1">
         <v>0</v>
@@ -6654,7 +6678,7 @@
         <v>637</v>
       </c>
       <c r="K83" t="s">
-        <v>784</v>
+        <v>988</v>
       </c>
       <c r="L83" s="1">
         <v>0</v>
@@ -6698,7 +6722,7 @@
         <v>638</v>
       </c>
       <c r="K84" t="s">
-        <v>785</v>
+        <v>989</v>
       </c>
       <c r="L84" s="1">
         <v>0</v>
@@ -6742,7 +6766,7 @@
         <v>639</v>
       </c>
       <c r="K85" t="s">
-        <v>786</v>
+        <v>988</v>
       </c>
       <c r="L85" s="1">
         <v>0</v>
@@ -9804,7 +9828,7 @@
         <v>694</v>
       </c>
       <c r="K155" t="s">
-        <v>841</v>
+        <v>990</v>
       </c>
       <c r="L155" s="1">
         <v>1</v>
@@ -9845,10 +9869,10 @@
         <v>583</v>
       </c>
       <c r="J156" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K156" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L156" s="1">
         <v>0</v>
@@ -9889,10 +9913,10 @@
         <v>583</v>
       </c>
       <c r="J157" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K157" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L157" s="1">
         <v>0</v>
@@ -9933,10 +9957,10 @@
         <v>583</v>
       </c>
       <c r="J158" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K158" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L158" s="1">
         <v>0</v>
@@ -9977,10 +10001,10 @@
         <v>583</v>
       </c>
       <c r="J159" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K159" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L159" s="1">
         <v>0</v>
@@ -10021,10 +10045,10 @@
         <v>583</v>
       </c>
       <c r="J160" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K160" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L160" s="1">
         <v>0</v>
@@ -10065,10 +10089,10 @@
         <v>583</v>
       </c>
       <c r="J161" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K161" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L161" s="1">
         <v>0</v>
@@ -10109,10 +10133,10 @@
         <v>583</v>
       </c>
       <c r="J162" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K162" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L162" s="1">
         <v>0</v>
@@ -10153,10 +10177,10 @@
         <v>583</v>
       </c>
       <c r="J163" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K163" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L163" s="1">
         <v>0</v>
@@ -10197,10 +10221,10 @@
         <v>583</v>
       </c>
       <c r="J164" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K164" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L164" s="1">
         <v>0</v>
@@ -10241,10 +10265,10 @@
         <v>583</v>
       </c>
       <c r="J165" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K165" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L165" s="1">
         <v>0</v>
@@ -10285,10 +10309,10 @@
         <v>583</v>
       </c>
       <c r="J166" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K166" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L166" s="1">
         <v>0</v>
@@ -10329,10 +10353,10 @@
         <v>583</v>
       </c>
       <c r="J167" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K167" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L167" s="1">
         <v>0</v>
@@ -10373,10 +10397,10 @@
         <v>583</v>
       </c>
       <c r="J168" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K168" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L168" s="1">
         <v>0</v>
@@ -10417,10 +10441,10 @@
         <v>583</v>
       </c>
       <c r="J169" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K169" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L169" s="1">
         <v>0</v>
@@ -10461,10 +10485,10 @@
         <v>583</v>
       </c>
       <c r="J170" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K170" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L170" s="1">
         <v>0</v>
@@ -10505,10 +10529,10 @@
         <v>583</v>
       </c>
       <c r="J171" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K171" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L171" s="1">
         <v>0</v>
@@ -10549,10 +10573,10 @@
         <v>583</v>
       </c>
       <c r="J172" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K172" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L172" s="1">
         <v>0</v>
@@ -10593,10 +10617,10 @@
         <v>583</v>
       </c>
       <c r="J173" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K173" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L173" s="1">
         <v>0</v>
@@ -10637,10 +10661,10 @@
         <v>583</v>
       </c>
       <c r="J174" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K174" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L174" s="1">
         <v>0</v>
@@ -10681,10 +10705,10 @@
         <v>583</v>
       </c>
       <c r="J175" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K175" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L175" s="1">
         <v>0</v>
@@ -10725,10 +10749,10 @@
         <v>583</v>
       </c>
       <c r="J176" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K176" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L176" s="1">
         <v>0</v>
@@ -10769,10 +10793,10 @@
         <v>583</v>
       </c>
       <c r="J177" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K177" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L177" s="1">
         <v>0</v>
@@ -10813,10 +10837,10 @@
         <v>583</v>
       </c>
       <c r="J178" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K178" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L178" s="1">
         <v>0</v>
@@ -10857,10 +10881,10 @@
         <v>583</v>
       </c>
       <c r="J179" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K179" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L179" s="1">
         <v>0</v>
@@ -10901,10 +10925,10 @@
         <v>583</v>
       </c>
       <c r="J180" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K180" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L180" s="1">
         <v>0</v>
@@ -10945,10 +10969,10 @@
         <v>583</v>
       </c>
       <c r="J181" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K181" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L181" s="1">
         <v>0</v>
@@ -10989,10 +11013,10 @@
         <v>583</v>
       </c>
       <c r="J182" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K182" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L182" s="1">
         <v>0</v>
@@ -11033,10 +11057,10 @@
         <v>583</v>
       </c>
       <c r="J183" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K183" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L183" s="1">
         <v>0</v>
@@ -11077,10 +11101,10 @@
         <v>583</v>
       </c>
       <c r="J184" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K184" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L184" s="1">
         <v>0</v>
@@ -11121,10 +11145,10 @@
         <v>583</v>
       </c>
       <c r="J185" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K185" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L185" s="1">
         <v>0</v>
@@ -11165,10 +11189,10 @@
         <v>583</v>
       </c>
       <c r="J186" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K186" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L186" s="1">
         <v>0</v>
@@ -11209,10 +11233,10 @@
         <v>583</v>
       </c>
       <c r="J187" t="s">
-        <v>695</v>
+        <v>994</v>
       </c>
       <c r="K187" t="s">
-        <v>842</v>
+        <v>994</v>
       </c>
       <c r="L187" s="1">
         <v>0</v>
@@ -11652,7 +11676,7 @@
         <v>698</v>
       </c>
       <c r="K197" t="s">
-        <v>845</v>
+        <v>993</v>
       </c>
       <c r="L197" s="1">
         <v>1</v>
@@ -11696,7 +11720,7 @@
         <v>698</v>
       </c>
       <c r="K198" t="s">
-        <v>845</v>
+        <v>993</v>
       </c>
       <c r="L198" s="1">
         <v>1</v>
@@ -11740,7 +11764,7 @@
         <v>698</v>
       </c>
       <c r="K199" t="s">
-        <v>845</v>
+        <v>993</v>
       </c>
       <c r="L199" s="1">
         <v>1</v>
@@ -11784,7 +11808,7 @@
         <v>698</v>
       </c>
       <c r="K200" t="s">
-        <v>845</v>
+        <v>993</v>
       </c>
       <c r="L200" s="1">
         <v>1</v>
@@ -11828,7 +11852,7 @@
         <v>698</v>
       </c>
       <c r="K201" t="s">
-        <v>845</v>
+        <v>993</v>
       </c>
       <c r="L201" s="1">
         <v>1</v>
@@ -11872,7 +11896,7 @@
         <v>698</v>
       </c>
       <c r="K202" t="s">
-        <v>845</v>
+        <v>993</v>
       </c>
       <c r="L202" s="1">
         <v>0</v>
@@ -11916,7 +11940,7 @@
         <v>698</v>
       </c>
       <c r="K203" t="s">
-        <v>845</v>
+        <v>993</v>
       </c>
       <c r="L203" s="1">
         <v>0</v>
@@ -12972,7 +12996,7 @@
         <v>705</v>
       </c>
       <c r="K227" t="s">
-        <v>852</v>
+        <v>990</v>
       </c>
       <c r="L227" s="1">
         <v>0</v>
@@ -13016,7 +13040,7 @@
         <v>705</v>
       </c>
       <c r="K228" t="s">
-        <v>852</v>
+        <v>990</v>
       </c>
       <c r="L228" s="1">
         <v>0</v>
@@ -14116,7 +14140,7 @@
         <v>726</v>
       </c>
       <c r="K253" t="s">
-        <v>873</v>
+        <v>988</v>
       </c>
       <c r="L253" s="1">
         <v>0</v>
@@ -14160,7 +14184,7 @@
         <v>726</v>
       </c>
       <c r="K254" t="s">
-        <v>873</v>
+        <v>988</v>
       </c>
       <c r="L254" s="1">
         <v>0</v>
@@ -14204,7 +14228,7 @@
         <v>726</v>
       </c>
       <c r="K255" t="s">
-        <v>873</v>
+        <v>988</v>
       </c>
       <c r="L255" s="1">
         <v>0</v>
@@ -14248,7 +14272,7 @@
         <v>727</v>
       </c>
       <c r="K256" t="s">
-        <v>874</v>
+        <v>727</v>
       </c>
       <c r="L256" s="1">
         <v>1</v>
@@ -14292,7 +14316,7 @@
         <v>727</v>
       </c>
       <c r="K257" t="s">
-        <v>874</v>
+        <v>727</v>
       </c>
       <c r="L257" s="1">
         <v>1</v>
@@ -14336,7 +14360,7 @@
         <v>727</v>
       </c>
       <c r="K258" t="s">
-        <v>874</v>
+        <v>727</v>
       </c>
       <c r="L258" s="1">
         <v>1</v>
@@ -14380,7 +14404,7 @@
         <v>727</v>
       </c>
       <c r="K259" t="s">
-        <v>874</v>
+        <v>727</v>
       </c>
       <c r="L259" s="1">
         <v>1</v>
@@ -14424,7 +14448,7 @@
         <v>728</v>
       </c>
       <c r="K260" t="s">
-        <v>875</v>
+        <v>989</v>
       </c>
       <c r="L260" s="1">
         <v>1</v>
@@ -14468,7 +14492,7 @@
         <v>728</v>
       </c>
       <c r="K261" t="s">
-        <v>875</v>
+        <v>989</v>
       </c>
       <c r="L261" s="1">
         <v>1</v>
@@ -15040,7 +15064,7 @@
         <v>730</v>
       </c>
       <c r="K274" t="s">
-        <v>877</v>
+        <v>989</v>
       </c>
       <c r="L274" s="1">
         <v>0</v>

</xml_diff>